<commit_message>
Align v0.3.2 locked validation release
</commit_message>
<xml_diff>
--- a/paper/Journal of Translational Medicine投稿/Additional_file_3_STROBE_TRIPOD_REMARK_checklists.xlsx
+++ b/paper/Journal of Translational Medicine投稿/Additional_file_3_STROBE_TRIPOD_REMARK_checklists.xlsx
@@ -576,7 +576,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Repository https://github.com/ahvsjags/EcoNiche-Opt; release tag v0.3.1-jtm-20260527; release archive https://github.com/ahvsjags/EcoNiche-Opt/archive/refs/tags/v0.3.1-jtm-20260527.zip.</t>
+          <t>Repository https://github.com/ahvsjags/EcoNiche-Opt; release tag v0.3.2-locked-validation-20260527; release archive https://github.com/ahvsjags/EcoNiche-Opt/archive/refs/tags/v0.3.2-locked-validation-20260527.zip.</t>
         </is>
       </c>
     </row>
@@ -593,7 +593,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Python package econiche_opt v0.3.1; R wrapper via reticulate; scripts listed in Code availability.</t>
+          <t>Python package econiche_opt v0.3.2; R wrapper via reticulate; scripts listed in Code availability.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
publish v0.3.4 public release assets
</commit_message>
<xml_diff>
--- a/paper/Journal of Translational Medicine投稿/Additional_file_3_STROBE_TRIPOD_REMARK_checklists.xlsx
+++ b/paper/Journal of Translational Medicine投稿/Additional_file_3_STROBE_TRIPOD_REMARK_checklists.xlsx
@@ -576,7 +576,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Repository https://github.com/ahvsjags/EcoNiche-Opt; release tag v0.3.2-locked-validation-20260527; release archive https://github.com/ahvsjags/EcoNiche-Opt/archive/refs/tags/v0.3.2-locked-validation-20260527.zip.</t>
+          <t>Repository https://github.com/ahvsjags/EcoNiche-Opt; release tag v0.3.4-gpu-lipid-pair-rescue-20260528; release archive https://github.com/ahvsjags/EcoNiche-Opt/archive/refs/tags/v0.3.4-gpu-lipid-pair-rescue-20260528.zip.</t>
         </is>
       </c>
     </row>
@@ -593,7 +593,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Python package econiche_opt v0.3.2; R wrapper via reticulate; scripts listed in Code availability.</t>
+          <t>Python package econiche_opt v0.3.4; R wrapper via reticulate; GPU biological-prior rescue and lipid/PI3K pair rescue packages and scripts listed in Code availability.</t>
         </is>
       </c>
     </row>

</xml_diff>